<commit_message>
Classificador: descritivo sem palavras repetidas em outra forma (TERMICA/TERMICO, ALADDIN/ALADIN)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/classificador/testes/sugestao_exemplo.xlsx
+++ b/classificador/testes/sugestao_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -978,6 +978,74 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17891108020591</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>{"GARRAFA TERMICA ALADIN TERMICO AZEITONA 1L CX C/6","GARRAFA TERMICA ALADDIN AZEITONA 1L","GARRAFA TERM ALADIM 1L"}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TERMICO PMI SA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ALADDIN</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>GARRAFA TERMICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>7891108020595</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>{"BISCOITO RECHEADO RECHEADA CHOCOLATE NESTLE NESTLLE 140G"}</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NESTLE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NESTLE</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>140</v>
+      </c>
+      <c r="G19" t="n">
+        <v>140</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>BISCOITO RECHEADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Classificador: descritivo + sugestões com UNIDADES SUGERIDA e CONTENIDO UNITARIO SUGERIDO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/classificador/testes/sugestao_exemplo.xlsx
+++ b/classificador/testes/sugestao_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1046,6 +1046,40 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>7891000100110</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>{"LEITE COND MOCA 12X395G","LEITE CONDENSADO MOCA 12X395G FARDO"}</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NESTLE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MOCA</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4740</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4740</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>LEITE CONDENSADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Classificador: descritivo + sugestões mantém gramatura em caixa (20X140G) e não sugere quantidade para caixa coerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/classificador/testes/sugestao_exemplo.xlsx
+++ b/classificador/testes/sugestao_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1080,6 +1080,74 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>57891095030014</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>{"BATATA PALHA YOKI TRADICIONAL 140G","BATATA PALHA YOKI 140G"}</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GENERAL MILLS</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>YOKI</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" t="n">
+        <v>140</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2800</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>BATATA PALHA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>7891095030017</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>{"BATATA PALHA YOKI TRADICIONAL 140G"}</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GENERAL MILLS</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>YOKI</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>140</v>
+      </c>
+      <c r="G22" t="n">
+        <v>140</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>BATATA PALHA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Classificador: descritivo mantém caractere especial da marca (M&M'S, L'OREAL, SCOTCH-BRITE, MAKE+)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/classificador/testes/sugestao_exemplo.xlsx
+++ b/classificador/testes/sugestao_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1148,6 +1148,74 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7891040000011</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>{"ESPONJA SCOTCH BRITE MULTIUSO C/3"}</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SCOTCH-BRITE</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ESPONJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7891040000013</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>{"CHOCOLATE M&amp;MS AMENDOIM 148G"}</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MARS</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>M&amp;M'S</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>148</v>
+      </c>
+      <c r="G24" t="n">
+        <v>148</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>CONFEITO DE CHOCOLATE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Classificador: COLORAU / COLORADO não são marca em tempero (marcaNaoCat por categoria)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/classificador/testes/sugestao_exemplo.xlsx
+++ b/classificador/testes/sugestao_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1216,6 +1216,70 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7890086510738</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>{"COLORAU BONZAO 80G","COLORADO BONZAO 80G"}</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ALFAPARF</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>COLORAU</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>80</v>
+      </c>
+      <c r="G25" t="n">
+        <v>80</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>TEMPERO NATURAL/ESPECIARIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>7898909893044</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>{"COLORADO NAZARE 1KG"}</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OUTRA MARCA</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>TEMPERO NATURAL/ESPECIARIA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>